<commit_message>
feat: Implement Reconciliation V2, refactor combined order workflows, and add registration kit inventory deduction. Uodate the unused to match start of day.
</commit_message>
<xml_diff>
--- a/backend/unused.xlsx
+++ b/backend/unused.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>TX ID</t>
   </si>
@@ -25,16 +25,7 @@
     <t>DATE</t>
   </si>
   <si>
-    <t>UABON3PL60</t>
-  </si>
-  <si>
-    <t>UAC1N3V6F1</t>
-  </si>
-  <si>
     <t>UAC9K3KFR4</t>
-  </si>
-  <si>
-    <t>UAEDI3TOLH</t>
   </si>
   <si>
     <t>UAF873RDZT</t>
@@ -46,7 +37,22 @@
     <t>UAFDC3X3SY</t>
   </si>
   <si>
-    <t>UAGB142ZSR</t>
+    <t>UAJB649XBD</t>
+  </si>
+  <si>
+    <t>UAKL54BNT3</t>
+  </si>
+  <si>
+    <t>UAK9O4EG8U</t>
+  </si>
+  <si>
+    <t>UAK6C43Y7F</t>
+  </si>
+  <si>
+    <t>UAK4S4BISY</t>
+  </si>
+  <si>
+    <t>UAKB64EU49</t>
   </si>
 </sst>
 </file>
@@ -55,13 +61,13 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="6">
     <numFmt numFmtId="176" formatCode="d/m"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="d/m/yy"/>
     <numFmt numFmtId="178" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="179" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -77,18 +83,31 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <sz val="10.5"/>
+      <color rgb="FF000000"/>
+      <name val="Liberation Mono"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -100,8 +119,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -109,6 +129,82 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -122,31 +218,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Arial"/>
@@ -154,75 +233,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -237,43 +249,121 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -285,19 +375,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -309,115 +429,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -428,6 +440,32 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -455,6 +493,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -466,50 +513,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -528,158 +531,168 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="179" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -942,7 +955,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultColWidth="12.6283185840708" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" customHeight="1" spans="1:3">
@@ -961,7 +974,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1">
-        <v>3240</v>
+        <v>1755</v>
       </c>
       <c r="C2" s="2"/>
     </row>
@@ -970,65 +983,73 @@
         <v>4</v>
       </c>
       <c r="B3" s="1">
-        <v>7830</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:3">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:2">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="1">
-        <v>1755</v>
-      </c>
-      <c r="C4" s="2"/>
+        <v>297</v>
+      </c>
     </row>
     <row r="5" customHeight="1" spans="1:2">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1">
-        <v>1755</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="6" customHeight="1" spans="1:2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1">
-        <v>386</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="7" customHeight="1" spans="1:2">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="1">
-        <v>297</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="1:2">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="1">
-        <v>2900</v>
+        <v>594</v>
       </c>
     </row>
     <row r="9" customHeight="1" spans="1:2">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="1">
-        <v>4954</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="10" customHeight="1" spans="1:2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-    </row>
-    <row r="11" customHeight="1" spans="1:2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
+      <c r="A10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1620</v>
+      </c>
+    </row>
+    <row r="11" customHeight="1" spans="1:3">
+      <c r="A11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="1">
+        <v>148</v>
+      </c>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" customHeight="1" spans="1:2">
       <c r="A12" s="1"/>
@@ -1042,10 +1063,9 @@
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
     </row>
-    <row r="15" customHeight="1" spans="1:3">
+    <row r="15" customHeight="1" spans="1:2">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="2"/>
     </row>
     <row r="16" customHeight="1" spans="1:2">
       <c r="A16" s="1"/>
@@ -1059,9 +1079,10 @@
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
     </row>
-    <row r="19" customHeight="1" spans="1:2">
+    <row r="19" customHeight="1" spans="1:3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" customHeight="1" spans="1:2">
       <c r="A20" s="1"/>
@@ -1071,14 +1092,14 @@
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
     </row>
-    <row r="22" customHeight="1" spans="1:2">
+    <row r="22" customHeight="1" spans="1:3">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
-    </row>
-    <row r="23" customHeight="1" spans="1:3">
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" customHeight="1" spans="1:2">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
-      <c r="C23" s="2"/>
     </row>
     <row r="24" customHeight="1" spans="1:2">
       <c r="A24" s="1"/>
@@ -1088,14 +1109,14 @@
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
     </row>
-    <row r="26" customHeight="1" spans="1:3">
+    <row r="26" customHeight="1" spans="1:2">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="2"/>
-    </row>
-    <row r="27" customHeight="1" spans="1:2">
+    </row>
+    <row r="27" customHeight="1" spans="1:3">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" customHeight="1" spans="1:2">
       <c r="A28" s="1"/>
@@ -1109,14 +1130,14 @@
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
     </row>
-    <row r="31" customHeight="1" spans="1:3">
+    <row r="31" customHeight="1" spans="1:2">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
-      <c r="C31" s="2"/>
-    </row>
-    <row r="32" customHeight="1" spans="1:2">
+    </row>
+    <row r="32" customHeight="1" spans="1:3">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" customHeight="1" spans="1:2">
       <c r="A33" s="1"/>
@@ -1130,14 +1151,14 @@
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
     </row>
-    <row r="36" customHeight="1" spans="1:3">
+    <row r="36" customHeight="1" spans="1:2">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
-      <c r="C36" s="2"/>
-    </row>
-    <row r="37" customHeight="1" spans="1:2">
+    </row>
+    <row r="37" customHeight="1" spans="1:3">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
+      <c r="C37" s="2"/>
     </row>
     <row r="38" customHeight="1" spans="1:2">
       <c r="A38" s="1"/>
@@ -1151,10 +1172,9 @@
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
     </row>
-    <row r="41" customHeight="1" spans="1:3">
+    <row r="41" customHeight="1" spans="1:2">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
-      <c r="C41" s="2"/>
     </row>
     <row r="42" customHeight="1" spans="1:2">
       <c r="A42" s="1"/>
@@ -1204,9 +1224,10 @@
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
     </row>
-    <row r="54" customHeight="1" spans="1:2">
+    <row r="54" customHeight="1" spans="1:3">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
+      <c r="C54" s="2"/>
     </row>
     <row r="55" customHeight="1" spans="1:2">
       <c r="A55" s="1"/>
@@ -1216,14 +1237,14 @@
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
     </row>
-    <row r="57" customHeight="1" spans="1:2">
+    <row r="57" customHeight="1" spans="1:3">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
-    </row>
-    <row r="58" customHeight="1" spans="1:3">
+      <c r="C57" s="2"/>
+    </row>
+    <row r="58" customHeight="1" spans="1:2">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
-      <c r="C58" s="2"/>
     </row>
     <row r="59" customHeight="1" spans="1:2">
       <c r="A59" s="1"/>
@@ -1250,22 +1271,23 @@
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
     </row>
-    <row r="65" customHeight="1" spans="1:3">
+    <row r="65" customHeight="1" spans="1:2">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
-      <c r="C65" s="2"/>
-    </row>
-    <row r="66" customHeight="1" spans="1:2">
+    </row>
+    <row r="66" customHeight="1" spans="1:3">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
+      <c r="C66" s="4"/>
     </row>
     <row r="67" customHeight="1" spans="1:2">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
     </row>
-    <row r="68" customHeight="1" spans="1:2">
+    <row r="68" customHeight="1" spans="1:3">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
+      <c r="C68" s="2"/>
     </row>
     <row r="69" customHeight="1" spans="1:2">
       <c r="A69" s="1"/>
@@ -1274,29 +1296,28 @@
     <row r="70" customHeight="1" spans="1:3">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
-      <c r="C70" s="3"/>
+      <c r="C70" s="2"/>
     </row>
     <row r="71" customHeight="1" spans="1:2">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
     </row>
-    <row r="72" customHeight="1" spans="1:3">
+    <row r="72" customHeight="1" spans="1:2">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
-      <c r="C72" s="2"/>
     </row>
     <row r="73" customHeight="1" spans="1:2">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
     </row>
-    <row r="74" customHeight="1" spans="1:3">
+    <row r="74" customHeight="1" spans="1:2">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
-      <c r="C74" s="2"/>
-    </row>
-    <row r="75" customHeight="1" spans="1:2">
+    </row>
+    <row r="75" customHeight="1" spans="1:3">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
+      <c r="C75" s="2"/>
     </row>
     <row r="76" customHeight="1" spans="1:2">
       <c r="A76" s="1"/>
@@ -1310,14 +1331,14 @@
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
     </row>
-    <row r="79" customHeight="1" spans="1:3">
+    <row r="79" customHeight="1" spans="1:2">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
-      <c r="C79" s="2"/>
-    </row>
-    <row r="80" customHeight="1" spans="1:2">
+    </row>
+    <row r="80" customHeight="1" spans="1:3">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
+      <c r="C80" s="2"/>
     </row>
     <row r="81" customHeight="1" spans="1:2">
       <c r="A81" s="1"/>
@@ -1331,10 +1352,9 @@
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
     </row>
-    <row r="84" customHeight="1" spans="1:3">
+    <row r="84" customHeight="1" spans="1:2">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
-      <c r="C84" s="2"/>
     </row>
     <row r="85" customHeight="1" spans="1:2">
       <c r="A85" s="1"/>
@@ -1351,22 +1371,6 @@
     <row r="88" customHeight="1" spans="1:2">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
-    </row>
-    <row r="89" customHeight="1" spans="1:2">
-      <c r="A89" s="1"/>
-      <c r="B89" s="1"/>
-    </row>
-    <row r="90" customHeight="1" spans="1:2">
-      <c r="A90" s="1"/>
-      <c r="B90" s="1"/>
-    </row>
-    <row r="91" customHeight="1" spans="1:2">
-      <c r="A91" s="1"/>
-      <c r="B91" s="1"/>
-    </row>
-    <row r="92" customHeight="1" spans="1:2">
-      <c r="A92" s="1"/>
-      <c r="B92" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>